<commit_message>
docs: add first-recorded dates to legacy KPI catalogue
</commit_message>
<xml_diff>
--- a/project X/configuration/Dashboard Legend.xlsx
+++ b/project X/configuration/Dashboard Legend.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RID" sheetId="1" r:id="R2cbda54bfa464d90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Definition" sheetId="2" r:id="R414e06d7dce34a49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Definition" sheetId="4" r:id="Rf23e02971a2f4e0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gold Source Coverage" sheetId="5" r:id="Rfc20f84c7c6b4dd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RID" sheetId="1" r:id="R6a84d481e5e1487b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Definition" sheetId="2" r:id="Rb976edc8087349a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Definition" sheetId="4" r:id="R37441d9bb1304a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gold Source Coverage" sheetId="5" r:id="R57645904a5e1403b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1832,6 +1832,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="dd mmm yyyy"/>
+  </x:numFmts>
   <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
@@ -1936,7 +1939,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="32">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2000,6 +2003,18 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="3">
@@ -5331,6 +5346,7 @@
     <x:col min="6" max="6" width="85" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="21" customWidth="1"/>
     <x:col min="8" max="8" width="28.54296875" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="2" customFormat="1" ht="30" customHeight="1">
@@ -5357,6 +5373,9 @@
       </x:c>
       <x:c r="H1" s="20" t="s">
         <x:v>256</x:v>
+      </x:c>
+      <x:c r="I1" s="20" t="str">
+        <x:v>Date Added</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="332" customHeight="1">
@@ -5399,6 +5418,9 @@
       </x:c>
       <x:c r="H2" s="13" t="s">
         <x:v>261</x:v>
+      </x:c>
+      <x:c r="I2" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="409" customHeight="1">
@@ -5449,6 +5471,9 @@
       <x:c r="H3" s="13" t="s">
         <x:v>266</x:v>
       </x:c>
+      <x:c r="I3" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="409" customHeight="1">
       <x:c r="A4" s="12" t="s">
@@ -5497,6 +5522,9 @@
       </x:c>
       <x:c r="H4" s="13" t="s">
         <x:v>261</x:v>
+      </x:c>
+      <x:c r="I4" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="409" customHeight="1">
@@ -5548,6 +5576,9 @@
       <x:c r="H5" s="13" t="s">
         <x:v>273</x:v>
       </x:c>
+      <x:c r="I5" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="409" customHeight="1">
       <x:c r="A6" s="12" t="s">
@@ -5598,6 +5629,9 @@
       <x:c r="H6" s="13" t="s">
         <x:v>273</x:v>
       </x:c>
+      <x:c r="I6" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="371" customHeight="1">
       <x:c r="A7" s="12" t="s">
@@ -5643,6 +5677,9 @@
       <x:c r="H7" s="13" t="s">
         <x:v>273</x:v>
       </x:c>
+      <x:c r="I7" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="371" customHeight="1">
       <x:c r="A8" s="12" t="s">
@@ -5688,6 +5725,9 @@
       <x:c r="H8" s="13" t="s">
         <x:v>266</x:v>
       </x:c>
+      <x:c r="I8" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="384" customHeight="1">
       <x:c r="A9" s="12" t="s">
@@ -5732,6 +5772,9 @@
       </x:c>
       <x:c r="H9" s="13" t="s">
         <x:v>266</x:v>
+      </x:c>
+      <x:c r="I9" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="409" customHeight="1">
@@ -5782,6 +5825,9 @@
       <x:c r="H10" s="13" t="s">
         <x:v>273</x:v>
       </x:c>
+      <x:c r="I10" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="319" customHeight="1">
       <x:c r="A11" s="12" t="s">
@@ -5823,6 +5869,9 @@
       </x:c>
       <x:c r="H11" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I11" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="409" customHeight="1">
@@ -5873,6 +5922,9 @@
       <x:c r="H12" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I12" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="215" customHeight="1">
       <x:c r="A13" s="12" t="s">
@@ -5905,6 +5957,9 @@
       </x:c>
       <x:c r="H13" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I13" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="371" customHeight="1">
@@ -5951,6 +6006,9 @@
       </x:c>
       <x:c r="H14" s="13" t="s">
         <x:v>273</x:v>
+      </x:c>
+      <x:c r="I14" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="409" customHeight="1">
@@ -6006,6 +6064,9 @@
       <x:c r="H15" s="13" t="s">
         <x:v>273</x:v>
       </x:c>
+      <x:c r="I15" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="358" customHeight="1">
       <x:c r="A16" s="12" t="s">
@@ -6047,6 +6108,9 @@
       <x:c r="H16" s="18" t="s">
         <x:v>291</x:v>
       </x:c>
+      <x:c r="I16" s="31" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="215" customHeight="1">
       <x:c r="A17" s="12" t="s">
@@ -6079,6 +6143,9 @@
       </x:c>
       <x:c r="H17" s="13" t="s">
         <x:v>266</x:v>
+      </x:c>
+      <x:c r="I17" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="384" customHeight="1">
@@ -6126,6 +6193,9 @@
       <x:c r="H18" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I18" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="306" customHeight="1">
       <x:c r="A19" s="12" t="s">
@@ -6168,6 +6238,9 @@
       <x:c r="H19" s="13" t="s">
         <x:v>320</x:v>
       </x:c>
+      <x:c r="I19" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="215" customHeight="1">
       <x:c r="A20" s="12" t="s">
@@ -6200,6 +6273,9 @@
       </x:c>
       <x:c r="H20" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I20" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="384" customHeight="1">
@@ -6247,6 +6323,9 @@
       <x:c r="H21" s="13" t="s">
         <x:v>329</x:v>
       </x:c>
+      <x:c r="I21" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="215" customHeight="1">
       <x:c r="A22" s="12" t="s">
@@ -6279,6 +6358,9 @@
       </x:c>
       <x:c r="H22" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I22" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="409" customHeight="1">
@@ -6327,6 +6409,9 @@
       </x:c>
       <x:c r="H23" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I23" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="409" customHeight="1">
@@ -6377,6 +6462,9 @@
       <x:c r="H24" s="18" t="s">
         <x:v>291</x:v>
       </x:c>
+      <x:c r="I24" s="31" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="215" customHeight="1">
       <x:c r="A25" s="12" t="s">
@@ -6409,6 +6497,9 @@
       </x:c>
       <x:c r="H25" s="13" t="s">
         <x:v>296</x:v>
+      </x:c>
+      <x:c r="I25" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="358" customHeight="1">
@@ -6453,6 +6544,9 @@
       <x:c r="H26" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I26" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="358" customHeight="1">
       <x:c r="A27" s="12" t="s">
@@ -6496,6 +6590,9 @@
       <x:c r="H27" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I27" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="358" customHeight="1">
       <x:c r="A28" s="12" t="s">
@@ -6538,6 +6635,9 @@
       </x:c>
       <x:c r="H28" s="13" t="s">
         <x:v>296</x:v>
+      </x:c>
+      <x:c r="I28" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="397" customHeight="1">
@@ -6586,6 +6686,9 @@
       <x:c r="H29" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I29" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="397" customHeight="1">
       <x:c r="A30" s="12" t="s">
@@ -6633,6 +6736,9 @@
       <x:c r="H30" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I30" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="345" customHeight="1">
       <x:c r="A31" s="12" t="s">
@@ -6676,6 +6782,9 @@
       <x:c r="H31" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I31" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="358" customHeight="1">
       <x:c r="A32" s="12" t="s">
@@ -6719,6 +6828,9 @@
       <x:c r="H32" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I32" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="345" customHeight="1">
       <x:c r="A33" s="12" t="s">
@@ -6761,6 +6873,9 @@
       </x:c>
       <x:c r="H33" s="13" t="s">
         <x:v>296</x:v>
+      </x:c>
+      <x:c r="I33" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="371" customHeight="1">
@@ -6807,6 +6922,9 @@
       <x:c r="H34" s="18" t="s">
         <x:v>291</x:v>
       </x:c>
+      <x:c r="I34" s="31" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="397" customHeight="1">
       <x:c r="A35" s="12" t="s">
@@ -6851,6 +6969,9 @@
       </x:c>
       <x:c r="H35" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I35" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="409" customHeight="1">
@@ -6902,6 +7023,9 @@
       <x:c r="H36" s="18" t="s">
         <x:v>291</x:v>
       </x:c>
+      <x:c r="I36" s="31" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="332" customHeight="1">
       <x:c r="A37" s="12" t="s">
@@ -6944,6 +7068,9 @@
       <x:c r="H37" s="13" t="s">
         <x:v>373</x:v>
       </x:c>
+      <x:c r="I37" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="215" customHeight="1">
       <x:c r="A38" s="12" t="s">
@@ -6976,6 +7103,9 @@
       </x:c>
       <x:c r="H38" s="13" t="s">
         <x:v>329</x:v>
+      </x:c>
+      <x:c r="I38" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="409" customHeight="1">
@@ -7020,6 +7150,9 @@
       <x:c r="H39" s="13" t="s">
         <x:v>329</x:v>
       </x:c>
+      <x:c r="I39" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="228" customHeight="1">
       <x:c r="A40" s="12" t="s">
@@ -7052,6 +7185,9 @@
       </x:c>
       <x:c r="H40" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I40" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="409" customHeight="1">
@@ -7100,6 +7236,9 @@
       <x:c r="H41" s="13" t="s">
         <x:v>266</x:v>
       </x:c>
+      <x:c r="I41" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="306" customHeight="1">
       <x:c r="A42" s="12" t="s">
@@ -7140,6 +7279,9 @@
       </x:c>
       <x:c r="H42" s="13" t="s">
         <x:v>329</x:v>
+      </x:c>
+      <x:c r="I42" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="345" customHeight="1">
@@ -7184,6 +7326,9 @@
       <x:c r="H43" s="13" t="s">
         <x:v>261</x:v>
       </x:c>
+      <x:c r="I43" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="306" customHeight="1">
       <x:c r="A44" s="12" t="s">
@@ -7225,6 +7370,9 @@
       </x:c>
       <x:c r="H44" s="13" t="s">
         <x:v>261</x:v>
+      </x:c>
+      <x:c r="I44" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="332" customHeight="1">
@@ -7268,6 +7416,9 @@
       </x:c>
       <x:c r="H45" s="13" t="s">
         <x:v>261</x:v>
+      </x:c>
+      <x:c r="I45" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="409" customHeight="1">
@@ -7317,6 +7468,9 @@
       <x:c r="H46" s="13" t="s">
         <x:v>261</x:v>
       </x:c>
+      <x:c r="I46" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="228" customHeight="1">
       <x:c r="A47" s="12" t="s">
@@ -7349,6 +7503,9 @@
       </x:c>
       <x:c r="H47" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I47" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="332" customHeight="1">
@@ -7392,6 +7549,9 @@
       </x:c>
       <x:c r="H48" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I48" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="358" customHeight="1">
@@ -7437,6 +7597,9 @@
       <x:c r="H49" s="13" t="s">
         <x:v>261</x:v>
       </x:c>
+      <x:c r="I49" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="319" customHeight="1">
       <x:c r="A50" s="12" t="s">
@@ -7478,6 +7641,9 @@
       </x:c>
       <x:c r="H50" s="13" t="s">
         <x:v>261</x:v>
+      </x:c>
+      <x:c r="I50" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="371" customHeight="1">
@@ -7524,6 +7690,9 @@
       </x:c>
       <x:c r="H51" s="13" t="s">
         <x:v>261</x:v>
+      </x:c>
+      <x:c r="I51" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="409" customHeight="1">
@@ -7573,6 +7742,9 @@
       <x:c r="H52" s="13" t="s">
         <x:v>261</x:v>
       </x:c>
+      <x:c r="I52" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="409" customHeight="1">
       <x:c r="A53" s="12" t="s">
@@ -7621,6 +7793,9 @@
       <x:c r="H53" s="13" t="s">
         <x:v>261</x:v>
       </x:c>
+      <x:c r="I53" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="319" customHeight="1">
       <x:c r="A54" s="12" t="s">
@@ -7660,6 +7835,9 @@
       </x:c>
       <x:c r="H54" s="13" t="s">
         <x:v>329</x:v>
+      </x:c>
+      <x:c r="I54" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="306" customHeight="1">
@@ -7703,6 +7881,9 @@
       <x:c r="H55" s="13" t="s">
         <x:v>320</x:v>
       </x:c>
+      <x:c r="I55" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="228" customHeight="1">
       <x:c r="A56" s="12" t="s">
@@ -7735,6 +7916,9 @@
       </x:c>
       <x:c r="H56" s="13" t="s">
         <x:v>320</x:v>
+      </x:c>
+      <x:c r="I56" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="332" customHeight="1">
@@ -7777,6 +7961,9 @@
       </x:c>
       <x:c r="H57" s="13" t="s">
         <x:v>373</x:v>
+      </x:c>
+      <x:c r="I57" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="345" customHeight="1">
@@ -7822,6 +8009,9 @@
       </x:c>
       <x:c r="H58" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I58" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="409" customHeight="1">
@@ -7874,6 +8064,9 @@
       <x:c r="H59" s="13" t="s">
         <x:v>273</x:v>
       </x:c>
+      <x:c r="I59" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="371" customHeight="1">
       <x:c r="A60" s="12" t="s">
@@ -7920,6 +8113,9 @@
       <x:c r="H60" s="13" t="s">
         <x:v>329</x:v>
       </x:c>
+      <x:c r="I60" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="332" customHeight="1">
       <x:c r="A61" s="12" t="s">
@@ -7963,6 +8159,9 @@
       <x:c r="H61" s="13" t="s">
         <x:v>266</x:v>
       </x:c>
+      <x:c r="I61" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="215" customHeight="1">
       <x:c r="A62" s="12" t="s">
@@ -7995,6 +8194,9 @@
       </x:c>
       <x:c r="H62" s="13" t="s">
         <x:v>266</x:v>
+      </x:c>
+      <x:c r="I62" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="397" customHeight="1">
@@ -8042,6 +8244,9 @@
       <x:c r="H63" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I63" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="371" customHeight="1">
       <x:c r="A64" s="12" t="s">
@@ -8085,6 +8290,9 @@
       </x:c>
       <x:c r="H64" s="13" t="s">
         <x:v>261</x:v>
+      </x:c>
+      <x:c r="I64" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="409" customHeight="1">
@@ -8134,6 +8342,9 @@
       <x:c r="H65" s="13" t="s">
         <x:v>273</x:v>
       </x:c>
+      <x:c r="I65" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="345" customHeight="1">
       <x:c r="A66" s="12" t="s">
@@ -8177,6 +8388,9 @@
       <x:c r="H66" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I66" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="332" customHeight="1">
       <x:c r="A67" s="12" t="s">
@@ -8219,6 +8433,9 @@
       <x:c r="H67" s="13" t="s">
         <x:v>266</x:v>
       </x:c>
+      <x:c r="I67" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="319" customHeight="1">
       <x:c r="A68" s="12" t="s">
@@ -8260,6 +8477,9 @@
       </x:c>
       <x:c r="H68" s="13" t="s">
         <x:v>261</x:v>
+      </x:c>
+      <x:c r="I68" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="409" customHeight="1">
@@ -8310,6 +8530,9 @@
       <x:c r="H69" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I69" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="332" customHeight="1">
       <x:c r="A70" s="12" t="s">
@@ -8352,6 +8575,9 @@
       <x:c r="H70" s="13" t="s">
         <x:v>373</x:v>
       </x:c>
+      <x:c r="I70" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="215" customHeight="1">
       <x:c r="A71" s="12" t="s">
@@ -8385,6 +8611,9 @@
       <x:c r="H71" s="18" t="s">
         <x:v>291</x:v>
       </x:c>
+      <x:c r="I71" s="31" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="241" customHeight="1">
       <x:c r="A72" s="12" t="s">
@@ -8417,6 +8646,9 @@
       </x:c>
       <x:c r="H72" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I72" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="384" customHeight="1">
@@ -8463,6 +8695,9 @@
       <x:c r="H73" s="13" t="s">
         <x:v>320</x:v>
       </x:c>
+      <x:c r="I73" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="228" customHeight="1">
       <x:c r="A74" s="12" t="s">
@@ -8495,6 +8730,9 @@
       </x:c>
       <x:c r="H74" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I74" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="371" customHeight="1">
@@ -8540,6 +8778,9 @@
       </x:c>
       <x:c r="H75" s="13" t="s">
         <x:v>273</x:v>
+      </x:c>
+      <x:c r="I75" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="409" customHeight="1">
@@ -8587,6 +8828,9 @@
       <x:c r="H76" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I76" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="371" customHeight="1">
       <x:c r="A77" s="12" t="s">
@@ -8629,6 +8873,9 @@
       </x:c>
       <x:c r="H77" s="13" t="s">
         <x:v>296</x:v>
+      </x:c>
+      <x:c r="I77" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="397" customHeight="1">
@@ -8676,6 +8923,9 @@
       <x:c r="H78" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I78" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" ht="409" customHeight="1">
       <x:c r="A79" s="12" t="s">
@@ -8722,6 +8972,9 @@
       <x:c r="H79" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I79" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="241" customHeight="1">
       <x:c r="A80" s="12" t="s">
@@ -8754,6 +9007,9 @@
       </x:c>
       <x:c r="H80" s="13" t="s">
         <x:v>296</x:v>
+      </x:c>
+      <x:c r="I80" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="358" customHeight="1">
@@ -8799,6 +9055,9 @@
       </x:c>
       <x:c r="H81" s="13" t="s">
         <x:v>495</x:v>
+      </x:c>
+      <x:c r="I81" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="409" customHeight="1">
@@ -8849,6 +9108,9 @@
       <x:c r="H82" s="18" t="s">
         <x:v>291</x:v>
       </x:c>
+      <x:c r="I82" s="31" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" ht="228" customHeight="1">
       <x:c r="A83" s="12" t="s">
@@ -8881,6 +9143,9 @@
       </x:c>
       <x:c r="H83" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I83" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="409" customHeight="1">
@@ -8930,6 +9195,9 @@
       <x:c r="H84" s="18" t="s">
         <x:v>291</x:v>
       </x:c>
+      <x:c r="I84" s="31" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="397" customHeight="1">
       <x:c r="A85" s="12" t="s">
@@ -8974,6 +9242,9 @@
       <x:c r="H85" s="13" t="s">
         <x:v>329</x:v>
       </x:c>
+      <x:c r="I85" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" ht="397" customHeight="1">
       <x:c r="A86" s="12" t="s">
@@ -9017,6 +9288,9 @@
       </x:c>
       <x:c r="H86" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I86" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="409" customHeight="1">
@@ -9064,6 +9338,9 @@
       <x:c r="H87" s="13" t="s">
         <x:v>296</x:v>
       </x:c>
+      <x:c r="I87" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="88" ht="409" customHeight="1">
       <x:c r="A88" s="12" t="s">
@@ -9106,6 +9383,9 @@
       </x:c>
       <x:c r="H88" s="13" t="s">
         <x:v>329</x:v>
+      </x:c>
+      <x:c r="I88" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="332" customHeight="1">
@@ -9151,6 +9431,9 @@
       <x:c r="H89" s="13" t="s">
         <x:v>329</x:v>
       </x:c>
+      <x:c r="I89" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="90" ht="332" customHeight="1">
       <x:c r="A90" s="12" t="s">
@@ -9195,6 +9478,9 @@
       <x:c r="H90" s="13" t="s">
         <x:v>329</x:v>
       </x:c>
+      <x:c r="I90" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="91" ht="228" customHeight="1">
       <x:c r="A91" s="12" t="s">
@@ -9227,6 +9513,9 @@
       </x:c>
       <x:c r="H91" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I91" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="332" customHeight="1">
@@ -9269,6 +9558,9 @@
       <x:c r="H92" s="13" t="s">
         <x:v>329</x:v>
       </x:c>
+      <x:c r="I92" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="93" ht="358" customHeight="1">
       <x:c r="A93" s="12" t="s">
@@ -9310,6 +9602,9 @@
       <x:c r="H93" s="18" t="s">
         <x:v>291</x:v>
       </x:c>
+      <x:c r="I93" s="31" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="94" ht="228" customHeight="1">
       <x:c r="A94" s="12" t="s">
@@ -9342,6 +9637,9 @@
       </x:c>
       <x:c r="H94" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I94" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="409" customHeight="1">
@@ -9391,6 +9689,9 @@
       <x:c r="H95" s="18" t="s">
         <x:v>291</x:v>
       </x:c>
+      <x:c r="I95" s="31" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="96" ht="228" customHeight="1">
       <x:c r="A96" s="12" t="s">
@@ -9423,6 +9724,9 @@
       </x:c>
       <x:c r="H96" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I96" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="371" customHeight="1">
@@ -9468,6 +9772,9 @@
       </x:c>
       <x:c r="H97" s="13" t="s">
         <x:v>373</x:v>
+      </x:c>
+      <x:c r="I97" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="409" customHeight="1">
@@ -9521,6 +9828,9 @@
       <x:c r="H98" s="13" t="s">
         <x:v>266</x:v>
       </x:c>
+      <x:c r="I98" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="99" ht="371" customHeight="1">
       <x:c r="A99" s="12" t="s">
@@ -9566,6 +9876,9 @@
       <x:c r="H99" s="13" t="s">
         <x:v>266</x:v>
       </x:c>
+      <x:c r="I99" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="100" ht="371" customHeight="1">
       <x:c r="A100" s="12" t="s">
@@ -9611,6 +9924,9 @@
       <x:c r="H100" s="13" t="s">
         <x:v>373</x:v>
       </x:c>
+      <x:c r="I100" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="101" ht="371" customHeight="1">
       <x:c r="A101" s="12" t="s">
@@ -9655,6 +9971,9 @@
       <x:c r="H101" s="13" t="s">
         <x:v>558</x:v>
       </x:c>
+      <x:c r="I101" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="102" ht="358" customHeight="1">
       <x:c r="A102" s="12" t="s">
@@ -9697,6 +10016,9 @@
       </x:c>
       <x:c r="H102" s="13" t="s">
         <x:v>558</x:v>
+      </x:c>
+      <x:c r="I102" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="371" customHeight="1">
@@ -9743,6 +10065,9 @@
       <x:c r="H103" s="13" t="s">
         <x:v>373</x:v>
       </x:c>
+      <x:c r="I103" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="104" ht="371" customHeight="1">
       <x:c r="A104" s="12" t="s">
@@ -9788,6 +10113,9 @@
       <x:c r="H104" s="13" t="s">
         <x:v>373</x:v>
       </x:c>
+      <x:c r="I104" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="105" ht="371" customHeight="1">
       <x:c r="A105" s="12" t="s">
@@ -9833,6 +10161,9 @@
       <x:c r="H105" s="13" t="s">
         <x:v>266</x:v>
       </x:c>
+      <x:c r="I105" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="106" ht="306" customHeight="1">
       <x:c r="A106" s="12" t="s">
@@ -9873,6 +10204,9 @@
       </x:c>
       <x:c r="H106" s="13" t="s">
         <x:v>329</x:v>
+      </x:c>
+      <x:c r="I106" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="409" customHeight="1">
@@ -9924,6 +10258,9 @@
       <x:c r="H107" s="13" t="s">
         <x:v>495</x:v>
       </x:c>
+      <x:c r="I107" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="108" ht="409" customHeight="1">
       <x:c r="A108" s="12" t="s">
@@ -9972,6 +10309,9 @@
       <x:c r="H108" s="13" t="s">
         <x:v>273</x:v>
       </x:c>
+      <x:c r="I108" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="109" ht="345" customHeight="1">
       <x:c r="A109" s="12" t="s">
@@ -10014,6 +10354,9 @@
       </x:c>
       <x:c r="H109" s="13" t="s">
         <x:v>261</x:v>
+      </x:c>
+      <x:c r="I109" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="332" customHeight="1">
@@ -10059,6 +10402,9 @@
       <x:c r="H110" s="13" t="s">
         <x:v>329</x:v>
       </x:c>
+      <x:c r="I110" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="111" ht="345" customHeight="1">
       <x:c r="A111" s="12" t="s">
@@ -10100,6 +10446,9 @@
       </x:c>
       <x:c r="H111" s="13" t="s">
         <x:v>373</x:v>
+      </x:c>
+      <x:c r="I111" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="384" customHeight="1">
@@ -10146,6 +10495,9 @@
       </x:c>
       <x:c r="H112" s="13" t="s">
         <x:v>495</x:v>
+      </x:c>
+      <x:c r="I112" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="409" customHeight="1">
@@ -10195,6 +10547,9 @@
       <x:c r="H113" s="13" t="s">
         <x:v>266</x:v>
       </x:c>
+      <x:c r="I113" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="114" ht="384" customHeight="1">
       <x:c r="A114" s="12" t="s">
@@ -10241,6 +10596,9 @@
       <x:c r="H114" s="13" t="s">
         <x:v>273</x:v>
       </x:c>
+      <x:c r="I114" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="115" ht="358" customHeight="1">
       <x:c r="A115" s="12" t="s">
@@ -10286,6 +10644,9 @@
       <x:c r="H115" s="13" t="s">
         <x:v>373</x:v>
       </x:c>
+      <x:c r="I115" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
     <x:row r="116" ht="202" customHeight="1">
       <x:c r="A116" s="12" t="s">
@@ -10318,6 +10679,9 @@
       </x:c>
       <x:c r="H116" s="13" t="s">
         <x:v>373</x:v>
+      </x:c>
+      <x:c r="I116" s="30" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="358" customHeight="1">
@@ -10363,6 +10727,9 @@
       </x:c>
       <x:c r="H117" s="18" t="s">
         <x:v>291</x:v>
+      </x:c>
+      <x:c r="I117" s="31" t="n">
+        <x:v>46260</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="409" customHeight="1">
@@ -10412,6 +10779,9 @@
       <x:c r="H118" s="13" t="s">
         <x:v>273</x:v>
       </x:c>
+      <x:c r="I118" s="30" t="n">
+        <x:v>46260</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -29202,12 +29572,12 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="6">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3cb4cf96aae491b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R860ec25cbe3c48df"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99fa784bf1e24ed4"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3928d7302fbb4a37"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c3590b9700d4443"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcfc9dd79477432c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d759c8da1b34a75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red294cea743b4417"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ba2bf85bb3b45e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4331134b4894fd9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35a692358f2e493c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3ee5d70f3b94a13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: append later Gold KPIs to the compatible definition sheet
</commit_message>
<xml_diff>
--- a/project X/configuration/Dashboard Legend.xlsx
+++ b/project X/configuration/Dashboard Legend.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RID" sheetId="1" r:id="R6a84d481e5e1487b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Definition" sheetId="2" r:id="Rb976edc8087349a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Definition" sheetId="4" r:id="R37441d9bb1304a9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gold Source Coverage" sheetId="5" r:id="R57645904a5e1403b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RID" sheetId="1" r:id="R2b29bc140ae54bfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Definition" sheetId="2" r:id="R0ce1f836c8ba43b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Definition" sheetId="4" r:id="Rb99f17245e72457b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gold Source Coverage" sheetId="5" r:id="Ra12edab3a1544aff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10783,6 +10783,1283 @@
         <x:v>46260</x:v>
       </x:c>
     </x:row>
+    <x:row r="119" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A119" s="13" t="str">
+        <x:v>GOLD-KPI-110</x:v>
+      </x:c>
+      <x:c r="B119" s="13" t="str">
+        <x:v>[R51]</x:v>
+      </x:c>
+      <x:c r="C119" s="13" t="str">
+        <x:v>Male Referrals</x:v>
+      </x:c>
+      <x:c r="D119" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E119" s="13" t="str">
+        <x:v>dim_person; fact_referral</x:v>
+      </x:c>
+      <x:c r="F119" s="13" t="str">
+        <x:v>Built; UAT pending. Gender-based referral analysis; reconcile unknowns and validate access controls.
+DAX / Python / Spark SQL:
+CALCULATE ( [Total Referrals], 'dim_person'[gender_clean] = "Male" )
+Python/Spark SQL: 05_gold_dimensions.py:194; 04_gold_model.py:232
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-male-referrals</x:v>
+      </x:c>
+      <x:c r="G119" s="13" t="str">
+        <x:v>Male Referrals</x:v>
+      </x:c>
+      <x:c r="H119" s="13" t="str">
+        <x:v>Section 9 - Other Measures</x:v>
+      </x:c>
+      <x:c r="I119" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A120" s="13" t="str">
+        <x:v>GOLD-KPI-111</x:v>
+      </x:c>
+      <x:c r="B120" s="13" t="str">
+        <x:v>[R51]</x:v>
+      </x:c>
+      <x:c r="C120" s="13" t="str">
+        <x:v>Female Referrals</x:v>
+      </x:c>
+      <x:c r="D120" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E120" s="13" t="str">
+        <x:v>dim_person; fact_referral</x:v>
+      </x:c>
+      <x:c r="F120" s="13" t="str">
+        <x:v>Built; UAT pending. Gender-based referral analysis; reconcile unknowns and validate access controls.
+DAX / Python / Spark SQL:
+CALCULATE ( [Total Referrals], 'dim_person'[gender_clean] = "Female" )
+Python/Spark SQL: 05_gold_dimensions.py:194; 04_gold_model.py:232
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-female-referrals</x:v>
+      </x:c>
+      <x:c r="G120" s="13" t="str">
+        <x:v>Female Referrals</x:v>
+      </x:c>
+      <x:c r="H120" s="13" t="str">
+        <x:v>Section 9 - Other Measures</x:v>
+      </x:c>
+      <x:c r="I120" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A121" s="13" t="str">
+        <x:v>GOLD-KPI-112</x:v>
+      </x:c>
+      <x:c r="B121" s="13" t="str">
+        <x:v>[R51]</x:v>
+      </x:c>
+      <x:c r="C121" s="13" t="str">
+        <x:v>Other Gender Referrals</x:v>
+      </x:c>
+      <x:c r="D121" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E121" s="13" t="str">
+        <x:v>dim_person; fact_referral</x:v>
+      </x:c>
+      <x:c r="F121" s="13" t="str">
+        <x:v>Built; UAT pending. Gender-based referral analysis; reconcile unknowns and validate access controls.
+DAX / Python / Spark SQL:
+CALCULATE ( [Total Referrals], 'dim_person'[gender_clean] = "Other" )
+Python/Spark SQL: 05_gold_dimensions.py:194; 04_gold_model.py:232
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-other-gender-referrals</x:v>
+      </x:c>
+      <x:c r="G121" s="13" t="str">
+        <x:v>Other Gender Referrals</x:v>
+      </x:c>
+      <x:c r="H121" s="13" t="str">
+        <x:v>Section 9 - Other Measures</x:v>
+      </x:c>
+      <x:c r="I121" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A122" s="13" t="str">
+        <x:v>GOLD-KPI-113</x:v>
+      </x:c>
+      <x:c r="B122" s="13" t="str">
+        <x:v>[R51]</x:v>
+      </x:c>
+      <x:c r="C122" s="13" t="str">
+        <x:v>Total Gendered Referrals</x:v>
+      </x:c>
+      <x:c r="D122" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E122" s="13" t="str">
+        <x:v>dim_person; fact_referral</x:v>
+      </x:c>
+      <x:c r="F122" s="13" t="str">
+        <x:v>Built; UAT pending. Gender-based referral analysis; reconcile unknowns and validate access controls.
+DAX / Python / Spark SQL:
+CALCULATE ( [Total Referrals], KEEPFILTERS ( FILTER ( 'dim_person', NOT ISBLANK ( 'dim_person'[gender_clean] ) &amp;&amp; 'dim_person'[gender_clean] &lt;&gt; "Unknown" ) ) )
+Python/Spark SQL: 05_gold_dimensions.py:194; 04_gold_model.py:232
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-total-gendered-referrals</x:v>
+      </x:c>
+      <x:c r="G122" s="13" t="str">
+        <x:v>Total Gendered Referrals</x:v>
+      </x:c>
+      <x:c r="H122" s="13" t="str">
+        <x:v>Section 9 - Other Measures</x:v>
+      </x:c>
+      <x:c r="I122" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A123" s="13" t="str">
+        <x:v>GOLD-KPI-114</x:v>
+      </x:c>
+      <x:c r="B123" s="13" t="str">
+        <x:v>[R15,R35,R62]</x:v>
+      </x:c>
+      <x:c r="C123" s="13" t="str">
+        <x:v>IPA Completed</x:v>
+      </x:c>
+      <x:c r="D123" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R15: Digital info &amp; signatures for IPA
+R35: Digitised IPA (review, approvals, signing, audit)
+R62: View completed placements, access IPAs, extract payment info</x:v>
+      </x:c>
+      <x:c r="E123" s="13" t="str">
+        <x:v>fact_ipa</x:v>
+      </x:c>
+      <x:c r="F123" s="13" t="str">
+        <x:v>Built; UAT pending. IPA-grain completion/signing backlog; completed includes closed signed records; pending excludes closed unsigned records.
+DAX / Python / Spark SQL:
+CALCULATE ( [IPAs Created], KEEPFILTERS ( 'fact_ipa'[is_ipa_completed] = TRUE () ) )
+Python/Spark SQL: 04_gold_model.py:817
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-ipa-completed</x:v>
+      </x:c>
+      <x:c r="G123" s="13" t="str">
+        <x:v>IPA Completed</x:v>
+      </x:c>
+      <x:c r="H123" s="13" t="str">
+        <x:v>Section 8 - IPA Measures</x:v>
+      </x:c>
+      <x:c r="I123" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A124" s="13" t="str">
+        <x:v>GOLD-KPI-115</x:v>
+      </x:c>
+      <x:c r="B124" s="13" t="str">
+        <x:v>[R15,R35,R62]</x:v>
+      </x:c>
+      <x:c r="C124" s="13" t="str">
+        <x:v>IPAs Pending Completion</x:v>
+      </x:c>
+      <x:c r="D124" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R15: Digital info &amp; signatures for IPA
+R35: Digitised IPA (review, approvals, signing, audit)
+R62: View completed placements, access IPAs, extract payment info</x:v>
+      </x:c>
+      <x:c r="E124" s="13" t="str">
+        <x:v>fact_ipa</x:v>
+      </x:c>
+      <x:c r="F124" s="13" t="str">
+        <x:v>Built; UAT pending. IPA-grain completion/signing backlog; completed includes closed signed records; pending excludes closed unsigned records.
+DAX / Python / Spark SQL:
+CALCULATE ( [IPAs Created], KEEPFILTERS ( 'fact_ipa'[is_ipa_pending] = TRUE () ) )
+Python/Spark SQL: 04_gold_model.py:817
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-ipas-pending-completion</x:v>
+      </x:c>
+      <x:c r="G124" s="13" t="str">
+        <x:v>IPAs Pending Completion</x:v>
+      </x:c>
+      <x:c r="H124" s="13" t="str">
+        <x:v>Section 8 - IPA Measures</x:v>
+      </x:c>
+      <x:c r="I124" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A125" s="13" t="str">
+        <x:v>GOLD-KPI-116</x:v>
+      </x:c>
+      <x:c r="B125" s="13" t="str">
+        <x:v>[R15,R35,R62]</x:v>
+      </x:c>
+      <x:c r="C125" s="13" t="str">
+        <x:v>IPAs Signed by Provider</x:v>
+      </x:c>
+      <x:c r="D125" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R15: Digital info &amp; signatures for IPA
+R35: Digitised IPA (review, approvals, signing, audit)
+R62: View completed placements, access IPAs, extract payment info</x:v>
+      </x:c>
+      <x:c r="E125" s="13" t="str">
+        <x:v>fact_ipa</x:v>
+      </x:c>
+      <x:c r="F125" s="13" t="str">
+        <x:v>Built; UAT pending. IPA-grain completion/signing backlog; completed includes closed signed records; pending excludes closed unsigned records.
+DAX / Python / Spark SQL:
+CALCULATE ( [IPAs Created], KEEPFILTERS ( 'fact_ipa'[signed_by_provider] = TRUE () ) )
+Python/Spark SQL: 04_gold_model.py:817
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-ipas-signed-by-provider</x:v>
+      </x:c>
+      <x:c r="G125" s="13" t="str">
+        <x:v>IPAs Signed by Provider</x:v>
+      </x:c>
+      <x:c r="H125" s="13" t="str">
+        <x:v>Section 8 - IPA Measures</x:v>
+      </x:c>
+      <x:c r="I125" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A126" s="13" t="str">
+        <x:v>GOLD-KPI-117</x:v>
+      </x:c>
+      <x:c r="B126" s="13" t="str">
+        <x:v>[R15,R35,R62]</x:v>
+      </x:c>
+      <x:c r="C126" s="13" t="str">
+        <x:v>IPAs Signed by Local Authority</x:v>
+      </x:c>
+      <x:c r="D126" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R15: Digital info &amp; signatures for IPA
+R35: Digitised IPA (review, approvals, signing, audit)
+R62: View completed placements, access IPAs, extract payment info</x:v>
+      </x:c>
+      <x:c r="E126" s="13" t="str">
+        <x:v>fact_ipa</x:v>
+      </x:c>
+      <x:c r="F126" s="13" t="str">
+        <x:v>Built; UAT pending. IPA-grain completion/signing backlog; completed includes closed signed records; pending excludes closed unsigned records.
+DAX / Python / Spark SQL:
+CALCULATE ( [IPAs Created], KEEPFILTERS ( 'fact_ipa'[signed_by_local_authority] = TRUE () ) )
+Python/Spark SQL: 04_gold_model.py:817
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-ipas-signed-by-local-authority</x:v>
+      </x:c>
+      <x:c r="G126" s="13" t="str">
+        <x:v>IPAs Signed by Local Authority</x:v>
+      </x:c>
+      <x:c r="H126" s="13" t="str">
+        <x:v>Section 8 - IPA Measures</x:v>
+      </x:c>
+      <x:c r="I126" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="132" hidden="0" customHeight="1">
+      <x:c r="A127" s="13" t="str">
+        <x:v>GOLD-KPI-118</x:v>
+      </x:c>
+      <x:c r="B127" s="13" t="str">
+        <x:v>[R24,R51,R52]</x:v>
+      </x:c>
+      <x:c r="C127" s="13" t="str">
+        <x:v>Snapshot referrals previous month</x:v>
+      </x:c>
+      <x:c r="D127" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R51: Robust data model: placement records, market intelligence, value analysis
+R52: Accurate and customisable reporting</x:v>
+      </x:c>
+      <x:c r="E127" s="13" t="str">
+        <x:v>dim_snapshot_month; fact_referral_snapshot</x:v>
+      </x:c>
+      <x:c r="F127" s="13" t="str">
+        <x:v>Built; UAT pending. Compare retained month-end state with the prior calendar month; missing prior data remains blank.
+DAX / Python / Spark SQL:
+VAR currentMonth = SELECTEDVALUE('dim_snapshot_month'[month_start])
+			RETURN IF(NOT ISBLANK(currentMonth), CALCULATE([Snapshot Referrals], REMOVEFILTERS('dim_snapshot_month'), 'dim_snapshot_month'[month_start] = EDATE(currentMonth,-1)))
+Python/Spark SQL: 05_gold_dimensions.py:390; 04_gold_model.py:567
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-snapshot-referrals-previous-month</x:v>
+      </x:c>
+      <x:c r="G127" s="13" t="str">
+        <x:v>Snapshot referrals previous month</x:v>
+      </x:c>
+      <x:c r="H127" s="13" t="str">
+        <x:v>Section 3 - Timebased</x:v>
+      </x:c>
+      <x:c r="I127" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="132" hidden="0" customHeight="1">
+      <x:c r="A128" s="13" t="str">
+        <x:v>GOLD-KPI-119</x:v>
+      </x:c>
+      <x:c r="B128" s="13" t="str">
+        <x:v>[R24,R51,R52]</x:v>
+      </x:c>
+      <x:c r="C128" s="13" t="str">
+        <x:v>Snapshot referrals MoM change</x:v>
+      </x:c>
+      <x:c r="D128" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R51: Robust data model: placement records, market intelligence, value analysis
+R52: Accurate and customisable reporting</x:v>
+      </x:c>
+      <x:c r="E128" s="13" t="str">
+        <x:v>dim_snapshot_month; fact_referral_snapshot</x:v>
+      </x:c>
+      <x:c r="F128" s="13" t="str">
+        <x:v>Built; UAT pending. Compare retained month-end state with the prior calendar month; missing prior data remains blank.
+DAX / Python / Spark SQL:
+VAR currentTotal = [Snapshot Referrals]
+			VAR previousTotal = [Snapshot referrals previous month]
+			RETURN IF(NOT ISBLANK(currentTotal) &amp;&amp; NOT ISBLANK(previousTotal), currentTotal - previousTotal)
+Python/Spark SQL: 04_gold_model.py:567; 05_gold_dimensions.py:390
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-snapshot-referrals-mom-change</x:v>
+      </x:c>
+      <x:c r="G128" s="13" t="str">
+        <x:v>Snapshot referrals MoM change</x:v>
+      </x:c>
+      <x:c r="H128" s="18" t="str">
+        <x:v>Section 3 - Timebased</x:v>
+      </x:c>
+      <x:c r="I128" s="31" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="132" hidden="0" customHeight="1">
+      <x:c r="A129" s="13" t="str">
+        <x:v>GOLD-KPI-120</x:v>
+      </x:c>
+      <x:c r="B129" s="13" t="str">
+        <x:v>[R24,R51,R52]</x:v>
+      </x:c>
+      <x:c r="C129" s="13" t="str">
+        <x:v>Snapshot referrals MoM percent</x:v>
+      </x:c>
+      <x:c r="D129" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R51: Robust data model: placement records, market intelligence, value analysis
+R52: Accurate and customisable reporting</x:v>
+      </x:c>
+      <x:c r="E129" s="13" t="str">
+        <x:v>dim_snapshot_month; fact_referral_snapshot</x:v>
+      </x:c>
+      <x:c r="F129" s="13" t="str">
+        <x:v>Built; UAT pending. Compare retained month-end state with the prior calendar month; missing prior data remains blank.
+DAX / Python / Spark SQL:
+DIVIDE([Snapshot referrals MoM change],[Snapshot referrals previous month])
+Python/Spark SQL: 04_gold_model.py:567; 05_gold_dimensions.py:390
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-snapshot-referrals-mom-percent</x:v>
+      </x:c>
+      <x:c r="G129" s="13" t="str">
+        <x:v>Snapshot referrals MoM percent</x:v>
+      </x:c>
+      <x:c r="H129" s="13" t="str">
+        <x:v>Section 3 - Timebased</x:v>
+      </x:c>
+      <x:c r="I129" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="132" hidden="0" customHeight="1">
+      <x:c r="A130" s="13" t="str">
+        <x:v>GOLD-KPI-121</x:v>
+      </x:c>
+      <x:c r="B130" s="13" t="str">
+        <x:v>[R24,R51]</x:v>
+      </x:c>
+      <x:c r="C130" s="13" t="str">
+        <x:v>Referrals closed during month</x:v>
+      </x:c>
+      <x:c r="D130" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E130" s="13" t="str">
+        <x:v>dim_date; fact_referral</x:v>
+      </x:c>
+      <x:c r="F130" s="13" t="str">
+        <x:v>Built; UAT pending. Distinct referrals by closure date in month; a flow measure, not closed state at snapshot. Closure date is derived.
+DAX / Python / Spark SQL:
+CALCULATE(DISTINCTCOUNT('fact_referral'[referral_id]), USERELATIONSHIP('fact_referral'[referral_closed_date],'dim_date'[date]), CROSSFILTER('fact_referral'[referral_created_date],'dim_date'[date],NONE), KEEPFILTERS(NOT ISBLANK('fact_referral'[referral_closed_date])))
+Python/Spark SQL: 05_gold_dimensions.py:128; 04_gold_model.py:232
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-referrals-closed-during-month</x:v>
+      </x:c>
+      <x:c r="G130" s="13" t="str">
+        <x:v>Referrals closed during month</x:v>
+      </x:c>
+      <x:c r="H130" s="18" t="str">
+        <x:v>Section 3 - Timebased</x:v>
+      </x:c>
+      <x:c r="I130" s="31" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A131" s="13" t="str">
+        <x:v>GOLD-KPI-122</x:v>
+      </x:c>
+      <x:c r="B131" s="13" t="str">
+        <x:v>[R13,R24,R25]</x:v>
+      </x:c>
+      <x:c r="C131" s="13" t="str">
+        <x:v>Matching referrals</x:v>
+      </x:c>
+      <x:c r="D131" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R13: Filter by specialisms, placement type, placement status
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R25: Quickly review detailed placement requests</x:v>
+      </x:c>
+      <x:c r="E131" s="13" t="str">
+        <x:v>Referral Category; bridge_referral_framework_category; fact_offer; fact_referral</x:v>
+      </x:c>
+      <x:c r="F131" s="13" t="str">
+        <x:v>Built; UAT pending. Distinct referrals after category and matching-offer filters; category totals are not additive.
+DAX / Python / Spark SQL:
+[Explorer referrals]
+Python/Spark SQL: 05_gold_dimensions.py:210; 04_gold_model.py:712; 04_gold_model.py:232
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-matching-referrals</x:v>
+      </x:c>
+      <x:c r="G131" s="13" t="str">
+        <x:v>Matching referrals</x:v>
+      </x:c>
+      <x:c r="H131" s="13" t="str">
+        <x:v>Section 1 - Referral Volume KPIs</x:v>
+      </x:c>
+      <x:c r="I131" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A132" s="13" t="str">
+        <x:v>GOLD-KPI-123</x:v>
+      </x:c>
+      <x:c r="B132" s="13" t="str">
+        <x:v>[R24,R25,R35,R51]</x:v>
+      </x:c>
+      <x:c r="C132" s="13" t="str">
+        <x:v>Journey referrals 1</x:v>
+      </x:c>
+      <x:c r="D132" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R25: Quickly review detailed placement requests
+R35: Digitised IPA (review, approvals, signing, audit)
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E132" s="13" t="str">
+        <x:v>Referral Category; bridge_referral_framework_category; fact_offer; fact_referral</x:v>
+      </x:c>
+      <x:c r="F132" s="13" t="str">
+        <x:v>Built; UAT pending. Referral created. One current stage per referral at refresh. Closed status overrides milestones; counts are not historic funnel conversion.
+DAX / Python / Spark SQL:
+COALESCE(CALCULATE([Matching referrals], KEEPFILTERS('fact_referral'[Journey stage order] = 1)), 0)
+Python/Spark SQL: 04_gold_model.py:232; 05_gold_dimensions.py:210; 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-referrals-1</x:v>
+      </x:c>
+      <x:c r="G132" s="13" t="str">
+        <x:v>Journey referrals 1</x:v>
+      </x:c>
+      <x:c r="H132" s="13" t="str">
+        <x:v>Section 1 - Referral Volume KPIs</x:v>
+      </x:c>
+      <x:c r="I132" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A133" s="13" t="str">
+        <x:v>GOLD-KPI-124</x:v>
+      </x:c>
+      <x:c r="B133" s="13" t="str">
+        <x:v>[R24,R25,R35,R51]</x:v>
+      </x:c>
+      <x:c r="C133" s="13" t="str">
+        <x:v>Journey referrals 2</x:v>
+      </x:c>
+      <x:c r="D133" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R25: Quickly review detailed placement requests
+R35: Digitised IPA (review, approvals, signing, audit)
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E133" s="13" t="str">
+        <x:v>Referral Category; bridge_referral_framework_category; fact_offer; fact_referral</x:v>
+      </x:c>
+      <x:c r="F133" s="13" t="str">
+        <x:v>Built; UAT pending. Provider search. One current stage per referral at refresh. Closed status overrides milestones; counts are not historic funnel conversion.
+DAX / Python / Spark SQL:
+COALESCE(CALCULATE([Matching referrals], KEEPFILTERS('fact_referral'[Journey stage order] = 2)), 0)
+Python/Spark SQL: 04_gold_model.py:232; 05_gold_dimensions.py:210; 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-referrals-2</x:v>
+      </x:c>
+      <x:c r="G133" s="13" t="str">
+        <x:v>Journey referrals 2</x:v>
+      </x:c>
+      <x:c r="H133" s="18" t="str">
+        <x:v>Section 1 - Referral Volume KPIs</x:v>
+      </x:c>
+      <x:c r="I133" s="31" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A134" s="13" t="str">
+        <x:v>GOLD-KPI-125</x:v>
+      </x:c>
+      <x:c r="B134" s="13" t="str">
+        <x:v>[R24,R25,R35,R51]</x:v>
+      </x:c>
+      <x:c r="C134" s="13" t="str">
+        <x:v>Journey referrals 3</x:v>
+      </x:c>
+      <x:c r="D134" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R25: Quickly review detailed placement requests
+R35: Digitised IPA (review, approvals, signing, audit)
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E134" s="13" t="str">
+        <x:v>Referral Category; bridge_referral_framework_category; fact_offer; fact_referral</x:v>
+      </x:c>
+      <x:c r="F134" s="13" t="str">
+        <x:v>Built; UAT pending. Offers received. One current stage per referral at refresh. Closed status overrides milestones; counts are not historic funnel conversion.
+DAX / Python / Spark SQL:
+COALESCE(CALCULATE([Matching referrals], KEEPFILTERS('fact_referral'[Journey stage order] = 3)), 0)
+Python/Spark SQL: 04_gold_model.py:232; 05_gold_dimensions.py:210; 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-referrals-3</x:v>
+      </x:c>
+      <x:c r="G134" s="13" t="str">
+        <x:v>Journey referrals 3</x:v>
+      </x:c>
+      <x:c r="H134" s="13" t="str">
+        <x:v>Section 1 - Referral Volume KPIs</x:v>
+      </x:c>
+      <x:c r="I134" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A135" s="13" t="str">
+        <x:v>GOLD-KPI-126</x:v>
+      </x:c>
+      <x:c r="B135" s="13" t="str">
+        <x:v>[R24,R25,R35,R51]</x:v>
+      </x:c>
+      <x:c r="C135" s="13" t="str">
+        <x:v>Journey referrals 4</x:v>
+      </x:c>
+      <x:c r="D135" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R25: Quickly review detailed placement requests
+R35: Digitised IPA (review, approvals, signing, audit)
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E135" s="13" t="str">
+        <x:v>Referral Category; bridge_referral_framework_category; fact_offer; fact_referral</x:v>
+      </x:c>
+      <x:c r="F135" s="13" t="str">
+        <x:v>Built; UAT pending. Offer accepted. One current stage per referral at refresh. Closed status overrides milestones; counts are not historic funnel conversion.
+DAX / Python / Spark SQL:
+COALESCE(CALCULATE([Matching referrals], KEEPFILTERS('fact_referral'[Journey stage order] = 4)), 0)
+Python/Spark SQL: 04_gold_model.py:232; 05_gold_dimensions.py:210; 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-referrals-4</x:v>
+      </x:c>
+      <x:c r="G135" s="13" t="str">
+        <x:v>Journey referrals 4</x:v>
+      </x:c>
+      <x:c r="H135" s="13" t="str">
+        <x:v>Section 1 - Referral Volume KPIs</x:v>
+      </x:c>
+      <x:c r="I135" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A136" s="13" t="str">
+        <x:v>GOLD-KPI-127</x:v>
+      </x:c>
+      <x:c r="B136" s="13" t="str">
+        <x:v>[R24,R25,R35,R51]</x:v>
+      </x:c>
+      <x:c r="C136" s="13" t="str">
+        <x:v>Journey referrals 5</x:v>
+      </x:c>
+      <x:c r="D136" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R25: Quickly review detailed placement requests
+R35: Digitised IPA (review, approvals, signing, audit)
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E136" s="13" t="str">
+        <x:v>Referral Category; bridge_referral_framework_category; fact_offer; fact_referral</x:v>
+      </x:c>
+      <x:c r="F136" s="13" t="str">
+        <x:v>Built; UAT pending. IPA created. One current stage per referral at refresh. Closed status overrides milestones; counts are not historic funnel conversion.
+DAX / Python / Spark SQL:
+COALESCE(CALCULATE([Matching referrals], KEEPFILTERS('fact_referral'[Journey stage order] = 5)), 0)
+Python/Spark SQL: 04_gold_model.py:232; 05_gold_dimensions.py:210; 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-referrals-5</x:v>
+      </x:c>
+      <x:c r="G136" s="13" t="str">
+        <x:v>Journey referrals 5</x:v>
+      </x:c>
+      <x:c r="H136" s="13" t="str">
+        <x:v>Section 1 - Referral Volume KPIs</x:v>
+      </x:c>
+      <x:c r="I136" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A137" s="13" t="str">
+        <x:v>GOLD-KPI-128</x:v>
+      </x:c>
+      <x:c r="B137" s="13" t="str">
+        <x:v>[R24,R25,R35,R51]</x:v>
+      </x:c>
+      <x:c r="C137" s="13" t="str">
+        <x:v>Journey referrals 6</x:v>
+      </x:c>
+      <x:c r="D137" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R25: Quickly review detailed placement requests
+R35: Digitised IPA (review, approvals, signing, audit)
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E137" s="13" t="str">
+        <x:v>Referral Category; bridge_referral_framework_category; fact_offer; fact_referral</x:v>
+      </x:c>
+      <x:c r="F137" s="13" t="str">
+        <x:v>Built; UAT pending. IPA signed. One current stage per referral at refresh. Closed status overrides milestones; counts are not historic funnel conversion.
+DAX / Python / Spark SQL:
+COALESCE(CALCULATE([Matching referrals], KEEPFILTERS('fact_referral'[Journey stage order] = 6)), 0)
+Python/Spark SQL: 04_gold_model.py:232; 05_gold_dimensions.py:210; 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-referrals-6</x:v>
+      </x:c>
+      <x:c r="G137" s="13" t="str">
+        <x:v>Journey referrals 6</x:v>
+      </x:c>
+      <x:c r="H137" s="18" t="str">
+        <x:v>Section 1 - Referral Volume KPIs</x:v>
+      </x:c>
+      <x:c r="I137" s="31" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A138" s="13" t="str">
+        <x:v>GOLD-KPI-129</x:v>
+      </x:c>
+      <x:c r="B138" s="13" t="str">
+        <x:v>[R24,R25,R35,R51]</x:v>
+      </x:c>
+      <x:c r="C138" s="13" t="str">
+        <x:v>Journey referrals 7</x:v>
+      </x:c>
+      <x:c r="D138" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R25: Quickly review detailed placement requests
+R35: Digitised IPA (review, approvals, signing, audit)
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E138" s="13" t="str">
+        <x:v>Referral Category; bridge_referral_framework_category; fact_offer; fact_referral</x:v>
+      </x:c>
+      <x:c r="F138" s="13" t="str">
+        <x:v>Built; UAT pending. Closed / cancelled / withdrawn. One current stage per referral at refresh. Closed status overrides milestones; counts are not historic funnel conversion.
+DAX / Python / Spark SQL:
+COALESCE(CALCULATE([Matching referrals], KEEPFILTERS('fact_referral'[Journey stage order] = 7)), 0)
+Python/Spark SQL: 04_gold_model.py:232; 05_gold_dimensions.py:210; 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-referrals-7</x:v>
+      </x:c>
+      <x:c r="G138" s="13" t="str">
+        <x:v>Journey referrals 7</x:v>
+      </x:c>
+      <x:c r="H138" s="13" t="str">
+        <x:v>Section 1 - Referral Volume KPIs</x:v>
+      </x:c>
+      <x:c r="I138" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A139" s="13" t="str">
+        <x:v>GOLD-KPI-130</x:v>
+      </x:c>
+      <x:c r="B139" s="13" t="str">
+        <x:v>[R24,R25,R35,R51]</x:v>
+      </x:c>
+      <x:c r="C139" s="13" t="str">
+        <x:v>Journey referrals 8</x:v>
+      </x:c>
+      <x:c r="D139" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R25: Quickly review detailed placement requests
+R35: Digitised IPA (review, approvals, signing, audit)
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E139" s="13" t="str">
+        <x:v>Referral Category; bridge_referral_framework_category; fact_offer; fact_referral</x:v>
+      </x:c>
+      <x:c r="F139" s="13" t="str">
+        <x:v>Built; UAT pending. Needs review. One current stage per referral at refresh. Closed status overrides milestones; counts are not historic funnel conversion.
+DAX / Python / Spark SQL:
+COALESCE(CALCULATE([Matching referrals], KEEPFILTERS('fact_referral'[Journey stage order] = 8)), 0)
+Python/Spark SQL: 04_gold_model.py:232; 05_gold_dimensions.py:210; 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-referrals-8</x:v>
+      </x:c>
+      <x:c r="G139" s="13" t="str">
+        <x:v>Journey referrals 8</x:v>
+      </x:c>
+      <x:c r="H139" s="18" t="str">
+        <x:v>Section 1 - Referral Volume KPIs</x:v>
+      </x:c>
+      <x:c r="I139" s="31" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="145.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A140" s="13" t="str">
+        <x:v>GOLD-KPI-131</x:v>
+      </x:c>
+      <x:c r="B140" s="13" t="str">
+        <x:v>[R24,R26,R28,R35]</x:v>
+      </x:c>
+      <x:c r="C140" s="13" t="str">
+        <x:v>Journey providers 0</x:v>
+      </x:c>
+      <x:c r="D140" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R26: Prioritise by match suitability, SOP, existing placements
+R28: Accept / reject / request further info
+R35: Digitised IPA (review, approvals, signing, audit)</x:v>
+      </x:c>
+      <x:c r="E140" s="13" t="str">
+        <x:v>dim_provider; dim_provider_home; fact_ipa; fact_offer</x:v>
+      </x:c>
+      <x:c r="F140" s="13" t="str">
+        <x:v>Built; UAT pending. Assigned / draft / unclear. Distinct provider at furthest evidenced stage in current cohort; not additive offer counts. No browsing evidence.
+DAX / Python / Spark SQL:
+COALESCE(COUNTROWS(FILTER(VALUES('dim_provider'[provider_id]), NOT ISBLANK('dim_provider'[provider_id]) &amp;&amp; CALCULATE([Provider matches offer status]) = 1 &amp;&amp; CALCULATE([Journey provider stage]) == 0)), 0)
+Python/Spark SQL: 05_gold_dimensions.py:155; 05_gold_dimensions.py:163; 04_gold_model.py:712; 05_gold_dimensions.py:253; 04_gold_model.py:817; 04_gold_model.py:847
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-providers-0</x:v>
+      </x:c>
+      <x:c r="G140" s="13" t="str">
+        <x:v>Journey providers 0</x:v>
+      </x:c>
+      <x:c r="H140" s="18" t="str">
+        <x:v>Section 2 - Provider Activity</x:v>
+      </x:c>
+      <x:c r="I140" s="31" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="145.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A141" s="13" t="str">
+        <x:v>GOLD-KPI-132</x:v>
+      </x:c>
+      <x:c r="B141" s="13" t="str">
+        <x:v>[R24,R26,R28,R35]</x:v>
+      </x:c>
+      <x:c r="C141" s="13" t="str">
+        <x:v>Journey providers 1</x:v>
+      </x:c>
+      <x:c r="D141" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R26: Prioritise by match suitability, SOP, existing placements
+R28: Accept / reject / request further info
+R35: Digitised IPA (review, approvals, signing, audit)</x:v>
+      </x:c>
+      <x:c r="E141" s="13" t="str">
+        <x:v>dim_provider; dim_provider_home; fact_ipa; fact_offer</x:v>
+      </x:c>
+      <x:c r="F141" s="13" t="str">
+        <x:v>Built; UAT pending. Message activity only. Distinct provider at furthest evidenced stage in current cohort; not additive offer counts. No browsing evidence.
+DAX / Python / Spark SQL:
+COALESCE(COUNTROWS(FILTER(VALUES('dim_provider'[provider_id]), NOT ISBLANK('dim_provider'[provider_id]) &amp;&amp; CALCULATE([Provider matches offer status]) = 1 &amp;&amp; CALCULATE([Journey provider stage]) == 1)), 0)
+Python/Spark SQL: 05_gold_dimensions.py:155; 05_gold_dimensions.py:163; 04_gold_model.py:712; 05_gold_dimensions.py:253; 04_gold_model.py:817; 04_gold_model.py:847
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-providers-1</x:v>
+      </x:c>
+      <x:c r="G141" s="13" t="str">
+        <x:v>Journey providers 1</x:v>
+      </x:c>
+      <x:c r="H141" s="18" t="str">
+        <x:v>Section 2 - Provider Activity</x:v>
+      </x:c>
+      <x:c r="I141" s="31" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="145.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A142" s="13" t="str">
+        <x:v>GOLD-KPI-133</x:v>
+      </x:c>
+      <x:c r="B142" s="13" t="str">
+        <x:v>[R24,R26,R28,R35]</x:v>
+      </x:c>
+      <x:c r="C142" s="13" t="str">
+        <x:v>Journey providers 2</x:v>
+      </x:c>
+      <x:c r="D142" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R26: Prioritise by match suitability, SOP, existing placements
+R28: Accept / reject / request further info
+R35: Digitised IPA (review, approvals, signing, audit)</x:v>
+      </x:c>
+      <x:c r="E142" s="13" t="str">
+        <x:v>dim_provider; dim_provider_home; fact_ipa; fact_offer</x:v>
+      </x:c>
+      <x:c r="F142" s="13" t="str">
+        <x:v>Built; UAT pending. Offers made. Distinct provider at furthest evidenced stage in current cohort; not additive offer counts. No browsing evidence.
+DAX / Python / Spark SQL:
+COALESCE(COUNTROWS(FILTER(VALUES('dim_provider'[provider_id]), NOT ISBLANK('dim_provider'[provider_id]) &amp;&amp; CALCULATE([Provider matches offer status]) = 1 &amp;&amp; CALCULATE([Journey provider stage]) == 2)), 0)
+Python/Spark SQL: 05_gold_dimensions.py:155; 05_gold_dimensions.py:163; 04_gold_model.py:712; 05_gold_dimensions.py:253; 04_gold_model.py:817; 04_gold_model.py:847
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-providers-2</x:v>
+      </x:c>
+      <x:c r="G142" s="13" t="str">
+        <x:v>Journey providers 2</x:v>
+      </x:c>
+      <x:c r="H142" s="13" t="str">
+        <x:v>Section 2 - Provider Activity</x:v>
+      </x:c>
+      <x:c r="I142" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="145.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A143" s="13" t="str">
+        <x:v>GOLD-KPI-134</x:v>
+      </x:c>
+      <x:c r="B143" s="13" t="str">
+        <x:v>[R24,R26,R28,R35]</x:v>
+      </x:c>
+      <x:c r="C143" s="13" t="str">
+        <x:v>Journey providers 3</x:v>
+      </x:c>
+      <x:c r="D143" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R26: Prioritise by match suitability, SOP, existing placements
+R28: Accept / reject / request further info
+R35: Digitised IPA (review, approvals, signing, audit)</x:v>
+      </x:c>
+      <x:c r="E143" s="13" t="str">
+        <x:v>dim_provider; dim_provider_home; fact_ipa; fact_offer</x:v>
+      </x:c>
+      <x:c r="F143" s="13" t="str">
+        <x:v>Built; UAT pending. Offer accepted. Distinct provider at furthest evidenced stage in current cohort; not additive offer counts. No browsing evidence.
+DAX / Python / Spark SQL:
+COALESCE(COUNTROWS(FILTER(VALUES('dim_provider'[provider_id]), NOT ISBLANK('dim_provider'[provider_id]) &amp;&amp; CALCULATE([Provider matches offer status]) = 1 &amp;&amp; CALCULATE([Journey provider stage]) == 3)), 0)
+Python/Spark SQL: 05_gold_dimensions.py:155; 05_gold_dimensions.py:163; 04_gold_model.py:712; 05_gold_dimensions.py:253; 04_gold_model.py:817; 04_gold_model.py:847
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-providers-3</x:v>
+      </x:c>
+      <x:c r="G143" s="13" t="str">
+        <x:v>Journey providers 3</x:v>
+      </x:c>
+      <x:c r="H143" s="13" t="str">
+        <x:v>Section 2 - Provider Activity</x:v>
+      </x:c>
+      <x:c r="I143" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="145.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A144" s="13" t="str">
+        <x:v>GOLD-KPI-135</x:v>
+      </x:c>
+      <x:c r="B144" s="13" t="str">
+        <x:v>[R24,R26,R28,R35]</x:v>
+      </x:c>
+      <x:c r="C144" s="13" t="str">
+        <x:v>Journey providers 5</x:v>
+      </x:c>
+      <x:c r="D144" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates
+R26: Prioritise by match suitability, SOP, existing placements
+R28: Accept / reject / request further info
+R35: Digitised IPA (review, approvals, signing, audit)</x:v>
+      </x:c>
+      <x:c r="E144" s="13" t="str">
+        <x:v>dim_provider; dim_provider_home; fact_ipa; fact_offer</x:v>
+      </x:c>
+      <x:c r="F144" s="13" t="str">
+        <x:v>Built; UAT pending. Provider signed. Distinct provider at furthest evidenced stage in current cohort; not additive offer counts. No browsing evidence.
+DAX / Python / Spark SQL:
+COALESCE(COUNTROWS(FILTER(VALUES('dim_provider'[provider_id]), NOT ISBLANK('dim_provider'[provider_id]) &amp;&amp; CALCULATE([Provider matches offer status]) = 1 &amp;&amp; CALCULATE([Journey provider stage]) == 5)), 0)
+Python/Spark SQL: 05_gold_dimensions.py:155; 05_gold_dimensions.py:163; 04_gold_model.py:712; 05_gold_dimensions.py:253; 04_gold_model.py:817; 04_gold_model.py:847
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-providers-5</x:v>
+      </x:c>
+      <x:c r="G144" s="13" t="str">
+        <x:v>Journey providers 5</x:v>
+      </x:c>
+      <x:c r="H144" s="13" t="str">
+        <x:v>Section 2 - Provider Activity</x:v>
+      </x:c>
+      <x:c r="I144" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A145" s="13" t="str">
+        <x:v>GOLD-KPI-136</x:v>
+      </x:c>
+      <x:c r="B145" s="13" t="str">
+        <x:v>[R35,R62]</x:v>
+      </x:c>
+      <x:c r="C145" s="13" t="str">
+        <x:v>Journey providers both signed</x:v>
+      </x:c>
+      <x:c r="D145" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R35: Digitised IPA (review, approvals, signing, audit)
+R62: View completed placements, access IPAs, extract payment info</x:v>
+      </x:c>
+      <x:c r="E145" s="13" t="str">
+        <x:v>dim_provider; fact_ipa; fact_offer</x:v>
+      </x:c>
+      <x:c r="F145" s="13" t="str">
+        <x:v>Built; UAT pending. Providers with both-signed IPA evidence; subset of provider-signed, not a further stage.
+DAX / Python / Spark SQL:
+COALESCE(COUNTROWS(FILTER(VALUES('dim_provider'[provider_id]),
+			VAR offerIDs = CALCULATETABLE(VALUES('fact_offer'[offer_id]))
+			VAR signedIPAs = CALCULATETABLE('fact_ipa', KEEPFILTERS(TREATAS(offerIDs, 'fact_ipa'[accepted_offer_id])))
+			RETURN NOT ISBLANK('dim_provider'[provider_id]) &amp;&amp; CALCULATE([Provider matches offer status]) = 1 &amp;&amp; COUNTROWS(FILTER(signedIPAs, 'fact_ipa'[signed_by_provider] == TRUE() &amp;&amp; 'fact_ipa'[signed_by_local_authority] == TRUE())) &gt; 0)),0)
+Python/Spark SQL: 05_gold_dimensions.py:155; 04_gold_model.py:817; 04_gold_model.py:712; 05_gold_dimensions.py:163
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-journey-providers-both-signed</x:v>
+      </x:c>
+      <x:c r="G145" s="13" t="str">
+        <x:v>Journey providers both signed</x:v>
+      </x:c>
+      <x:c r="H145" s="13" t="str">
+        <x:v>Section 2 - Provider Activity</x:v>
+      </x:c>
+      <x:c r="I145" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A146" s="13" t="str">
+        <x:v>GOLD-KPI-137</x:v>
+      </x:c>
+      <x:c r="B146" s="13" t="str">
+        <x:v>[R26,R51]</x:v>
+      </x:c>
+      <x:c r="C146" s="13" t="str">
+        <x:v>Provider Response Rate</x:v>
+      </x:c>
+      <x:c r="D146" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R26: Prioritise by match suitability, SOP, existing placements
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E146" s="13" t="str">
+        <x:v>fact_provider_kpi_monthly</x:v>
+      </x:c>
+      <x:c r="F146" s="13" t="str">
+        <x:v>Built; UAT pending. Assignment-cohort component based on qualifying offers/reasons. Not a message SLA, composite score or suitability rating.
+DAX / Python / Spark SQL:
+DIVIDE ( [Provider Qualifying Responses], [Provider Response Opportunities] )
+Python/Spark SQL: 04_gold_model.py:935
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-provider-response-rate</x:v>
+      </x:c>
+      <x:c r="G146" s="13" t="str">
+        <x:v>Provider Response Rate</x:v>
+      </x:c>
+      <x:c r="H146" s="13" t="str">
+        <x:v>Section 2 - Provider Activity</x:v>
+      </x:c>
+      <x:c r="I146" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="184.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A147" s="13" t="str">
+        <x:v>GOLD-KPI-138</x:v>
+      </x:c>
+      <x:c r="B147" s="13" t="str">
+        <x:v>[R26,R51]</x:v>
+      </x:c>
+      <x:c r="C147" s="13" t="str">
+        <x:v>Provider Average Response Hours</x:v>
+      </x:c>
+      <x:c r="D147" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R26: Prioritise by match suitability, SOP, existing placements
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E147" s="13" t="str">
+        <x:v>fact_provider_kpi_monthly</x:v>
+      </x:c>
+      <x:c r="F147" s="13" t="str">
+        <x:v>Built; UAT pending. Assignment-cohort component based on qualifying offers/reasons. Not a message SLA, composite score or suitability rating.
+DAX / Python / Spark SQL:
+DIVIDE (
+				SUMX (
+					'fact_provider_kpi_monthly',
+					'fact_provider_kpi_monthly'[average_response_minutes]
+						* 'fact_provider_kpi_monthly'[qualifying_response_count]
+				),
+				[Provider Qualifying Responses] * 60
+			)
+Python/Spark SQL: 04_gold_model.py:935
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-provider-average-response-hours</x:v>
+      </x:c>
+      <x:c r="G147" s="13" t="str">
+        <x:v>Provider Average Response Hours</x:v>
+      </x:c>
+      <x:c r="H147" s="13" t="str">
+        <x:v>Section 2 - Provider Activity</x:v>
+      </x:c>
+      <x:c r="I147" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="132" hidden="0" customHeight="1">
+      <x:c r="A148" s="13" t="str">
+        <x:v>GOLD-KPI-139</x:v>
+      </x:c>
+      <x:c r="B148" s="13" t="str">
+        <x:v>[R26,R51]</x:v>
+      </x:c>
+      <x:c r="C148" s="13" t="str">
+        <x:v>Provider Offer Conversion Rate</x:v>
+      </x:c>
+      <x:c r="D148" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R26: Prioritise by match suitability, SOP, existing placements
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E148" s="13" t="str">
+        <x:v>fact_provider_kpi_monthly</x:v>
+      </x:c>
+      <x:c r="F148" s="13" t="str">
+        <x:v>Built; UAT pending. Assignment-cohort component based on qualifying offers/reasons. Not a message SLA, composite score or suitability rating.
+DAX / Python / Spark SQL:
+DIVIDE (
+				SUM ( 'fact_provider_kpi_monthly'[accepted_offer_count] ),
+				SUM ( 'fact_provider_kpi_monthly'[offers_submitted_count] )
+			)
+Python/Spark SQL: 04_gold_model.py:935
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-provider-offer-conversion-rate</x:v>
+      </x:c>
+      <x:c r="G148" s="13" t="str">
+        <x:v>Provider Offer Conversion Rate</x:v>
+      </x:c>
+      <x:c r="H148" s="13" t="str">
+        <x:v>Section 2 - Provider Activity</x:v>
+      </x:c>
+      <x:c r="I148" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="132" hidden="0" customHeight="1">
+      <x:c r="A149" s="13" t="str">
+        <x:v>GOLD-KPI-140</x:v>
+      </x:c>
+      <x:c r="B149" s="13" t="str">
+        <x:v>[R26,R51]</x:v>
+      </x:c>
+      <x:c r="C149" s="13" t="str">
+        <x:v>Provider Target Placement Rate</x:v>
+      </x:c>
+      <x:c r="D149" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R26: Prioritise by match suitability, SOP, existing placements
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E149" s="13" t="str">
+        <x:v>fact_provider_kpi_monthly</x:v>
+      </x:c>
+      <x:c r="F149" s="13" t="str">
+        <x:v>Built; UAT pending. Assignment-cohort component based on qualifying offers/reasons. Not a message SLA, composite score or suitability rating.
+DAX / Python / Spark SQL:
+DIVIDE (
+				SUM ( 'fact_provider_kpi_monthly'[placed_by_target_count] ),
+				SUM ( 'fact_provider_kpi_monthly'[successful_referral_count] )
+			)
+Python/Spark SQL: 04_gold_model.py:935
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-provider-target-placement-rate</x:v>
+      </x:c>
+      <x:c r="G149" s="13" t="str">
+        <x:v>Provider Target Placement Rate</x:v>
+      </x:c>
+      <x:c r="H149" s="13" t="str">
+        <x:v>Section 2 - Provider Activity</x:v>
+      </x:c>
+      <x:c r="I149" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A150" s="13" t="str">
+        <x:v>GOLD-KPI-141</x:v>
+      </x:c>
+      <x:c r="B150" s="13" t="str">
+        <x:v>[R13,R51]</x:v>
+      </x:c>
+      <x:c r="C150" s="13" t="str">
+        <x:v>Preferred-city distance coverage</x:v>
+      </x:c>
+      <x:c r="D150" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R13: Filter by specialisms, placement type, placement status
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E150" s="13" t="str">
+        <x:v>fact_offer</x:v>
+      </x:c>
+      <x:c r="F150" s="13" t="str">
+        <x:v>Built; UAT pending. Share of offers with preference-city distance evidence. Missing coordinates are not zero distance.
+DAX / Python / Spark SQL:
+DIVIDE([Offers with preferred-city distance],[Offers Submitted])
+Python/Spark SQL: 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-preferred-city-distance-coverage</x:v>
+      </x:c>
+      <x:c r="G150" s="13" t="str">
+        <x:v>Preferred-city distance coverage</x:v>
+      </x:c>
+      <x:c r="H150" s="13" t="str">
+        <x:v>Section 9 - Other Measures</x:v>
+      </x:c>
+      <x:c r="I150" s="30" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A151" s="13" t="str">
+        <x:v>GOLD-KPI-142</x:v>
+      </x:c>
+      <x:c r="B151" s="13" t="str">
+        <x:v>[R13,R51]</x:v>
+      </x:c>
+      <x:c r="C151" s="13" t="str">
+        <x:v>Median preferred-city distance km</x:v>
+      </x:c>
+      <x:c r="D151" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R13: Filter by specialisms, placement type, placement status
+R51: Robust data model: placement records, market intelligence, value analysis</x:v>
+      </x:c>
+      <x:c r="E151" s="13" t="str">
+        <x:v>fact_offer</x:v>
+      </x:c>
+      <x:c r="F151" s="13" t="str">
+        <x:v>Built; UAT pending. City-centroid to postcode straight-line estimate, not child-address or road distance; approved coordinates required.
+DAX / Python / Spark SQL:
+MEDIANX(FILTER('fact_offer','fact_offer'[referral_to_home_distance_status]="APPROXIMATE_PREFERENCE_CITY" &amp;&amp; NOT ISBLANK('fact_offer'[referral_to_home_distance_km])),'fact_offer'[referral_to_home_distance_km])
+Python/Spark SQL: 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-median-preferred-city-distance-km</x:v>
+      </x:c>
+      <x:c r="G151" s="13" t="str">
+        <x:v>Median preferred-city distance km</x:v>
+      </x:c>
+      <x:c r="H151" s="18" t="str">
+        <x:v>Section 9 - Other Measures</x:v>
+      </x:c>
+      <x:c r="I151" s="31" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A152" s="13" t="str">
+        <x:v>GOLD-KPI-143</x:v>
+      </x:c>
+      <x:c r="B152" s="13" t="str">
+        <x:v>[R26,R51,R93]</x:v>
+      </x:c>
+      <x:c r="C152" s="13" t="str">
+        <x:v>Homes Offered</x:v>
+      </x:c>
+      <x:c r="D152" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R26: Prioritise by match suitability, SOP, existing placements
+R51: Robust data model: placement records, market intelligence, value analysis
+R93: Placement officer: provider directory, services, homes, docs</x:v>
+      </x:c>
+      <x:c r="E152" s="13" t="str">
+        <x:v>fact_offer</x:v>
+      </x:c>
+      <x:c r="F152" s="13" t="str">
+        <x:v>Built; UAT pending. Distinct offered homes in current context; not spare capacity or available beds.
+DAX / Python / Spark SQL:
+CALCULATE ( DISTINCTCOUNT ( 'fact_offer'[provider_home_id] ),
+			    KEEPFILTERS ( FILTER ( 'fact_offer', NOT ISBLANK ( 'fact_offer'[provider_home_id] ) &amp;&amp; 'fact_offer'[provider_home_id] &lt;&gt; "" ) ) )
+Python/Spark SQL: 04_gold_model.py:712
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-homes-offered</x:v>
+      </x:c>
+      <x:c r="G152" s="13" t="str">
+        <x:v>Homes Offered</x:v>
+      </x:c>
+      <x:c r="H152" s="18" t="str">
+        <x:v>Section 6 - Provider Registry</x:v>
+      </x:c>
+      <x:c r="I152" s="31" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A153" s="13" t="str">
+        <x:v>GOLD-KPI-144</x:v>
+      </x:c>
+      <x:c r="B153" s="13" t="str">
+        <x:v>[R16,R24]</x:v>
+      </x:c>
+      <x:c r="C153" s="13" t="str">
+        <x:v>Critical Overdue Referrals</x:v>
+      </x:c>
+      <x:c r="D153" s="13" t="str">
+        <x:v>Proposed requirement association; owner approval pending.
+R16: Priority information flagged in placement requests
+R24: Dashboard: status overview, provider updates, task mgmt, quick updates</x:v>
+      </x:c>
+      <x:c r="E153" s="13" t="str">
+        <x:v>fact_referral</x:v>
+      </x:c>
+      <x:c r="F153" s="13" t="str">
+        <x:v>Built; UAT pending. Operational overdue/critical cohort; validate urgency rule with owner before escalation.
+DAX / Python / Spark SQL:
+CALCULATE ( [Open Overdue Referrals],
+			    KEEPFILTERS ( 'fact_referral'[placement_urgency_band] = "Critical" ) )
+Python/Spark SQL: 04_gold_model.py:232
+Full logic: KPI_CALCULATION_TRACEABILITY.md#dax-business-critical-overdue-referrals</x:v>
+      </x:c>
+      <x:c r="G153" s="13" t="str">
+        <x:v>Critical Overdue Referrals</x:v>
+      </x:c>
+      <x:c r="H153" s="18" t="str">
+        <x:v>Section 1 - Referral Volume KPIs</x:v>
+      </x:c>
+      <x:c r="I153" s="31" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -29572,12 +30849,12 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="6">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d759c8da1b34a75"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red294cea743b4417"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ba2bf85bb3b45e2"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4331134b4894fd9"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35a692358f2e493c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3ee5d70f3b94a13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re15c6671166c4430"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93d092c2e3524c30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a6cd2630c194579"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d78befe167c48f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re01f66f172734980"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R665e656d83d946e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>